<commit_message>
update Simplified Publish d85202ee94f251afc0b0fb97baa620535afd14a0
</commit_message>
<xml_diff>
--- a/cp-card-custodian/ig/StructureDefinition-pdsm-simplified-publish.xlsx
+++ b/cp-card-custodian/ig/StructureDefinition-pdsm-simplified-publish.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-05T16:17:29+00:00</t>
+    <t>2026-05-06T12:21:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -991,7 +991,7 @@
 </t>
   </si>
   <si>
-    <t>Organization which maintains the document</t>
+    <t>Organisme responsable de la gestion du document. Information transmise dans le VIHF.</t>
   </si>
   <si>
     <t>Identifies the organization or group who is responsible for ongoing maintenance of and access to the document.</t>
@@ -5470,7 +5470,7 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G29" t="s" s="2">
         <v>93</v>

</xml_diff>